<commit_message>
refactor into 3 projects
</commit_message>
<xml_diff>
--- a/LlmMoveiAgentResults.xlsx
+++ b/LlmMoveiAgentResults.xlsx
@@ -15,8 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -76,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -105,6 +106,7 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -524,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ42"/>
+  <dimension ref="A1:AJ45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" style="7" min="1" max="1"/>
@@ -2262,7 +2264,7 @@
       </c>
       <c r="AJ15" s="8" t="inlineStr">
         <is>
-          <t>Verified, and worse than it looks — strict 3/42, answered 0 of 34. Made ZERO real tool calls in all 42 runs: it prints tool calls as prose ('&lt;|tool call{...}|&gt;' and json blocks) in 17 runs instead of using the tool-call channel. Re-ran with wire capture: 25 tool definitions were sent correctly and it described them accurately, then called none — model behaviour, not a harness fault. Its 4 'correct' include 2 grader false positives. Belongs with the hard fails.</t>
+          <t>HARD FAIL — zero tool calls in all 42 runs, wire-confirmed. Strict 3/42 and answered 0 of 34. It prints tool calls as prose ('&lt;|tool call{...}|&gt;' and json blocks) in 17 runs instead of using the tool-call channel. Re-ran with wire capture: 25 tool definitions were sent correctly and it described them accurately, then called none — model behaviour, not a harness fault. Its 4 'correct' include 2 grader false positives. The numbers here are real but should be read as a hard fail, not a low score.</t>
         </is>
       </c>
     </row>
@@ -2384,7 +2386,7 @@
       </c>
       <c r="AJ16" s="8" t="inlineStr">
         <is>
-          <t>Verified. Strict 8/42 — but all 8 are refusals; it answered 0 of 34. Zero tool calls in all 42 runs and refuses 33 of 34 answerable questions ('I don't have access to information about...'). Wire capture confirms 25 tools were sent and none called. Its perfect 8/8 refusal score is the clearest demonstration here that refusal accuracy is meaningless without the over-refusal denominator. Belongs with the hard fails.</t>
+          <t>HARD FAIL — zero tool calls in all 42 runs, wire-confirmed (25 tools sent, none called). Strict 8/42, but all 8 are refusals; it answered 0 of 34 and refused 33 of 34 answerable questions ('I don't have access to information about...'). Its perfect 8/8 refusal score is the clearest demonstration here that refusal accuracy is meaningless without the over-refusal denominator.</t>
         </is>
       </c>
     </row>
@@ -2867,7 +2869,129 @@
       </c>
       <c r="AJ20" s="8" t="inlineStr">
         <is>
-          <t>Verified. Strict 1/42. CORRECTION to an earlier note: that single point is NOT a truncation artefact — the run finished with finish_reason 'stop' and a complete sentence. It is a different false positive: the model narrates a plan it never executes ('I am calling search_films_by_title...') and the conditional phrase 'I cannot proceed further without guessing' trips the refusal classifier. Still unfixed. Ignored Agent:Thinking=false entirely (reasoning in 42/42 iterations) and burned the whole 2500-token cap in 31/42 runs, giving 31 empty answers and zero tool calls for the sweep. Mean 2298 output tokens vs ~100 elsewhere; 26 min wall clock. Untestable at this MaxOutputTokens rather than proven bad.</t>
+          <t>HARD FAIL — zero tool calls, wire-confirmed, at BOTH token caps. Strict 1/42 and its true score is 0: the single point is a grader artefact (a complete sentence containing the conditional 'I cannot proceed further without guessing', inside a plan it never executed, read as a refusal). RETEST: re-run at MaxOutputTokens 6000 (runs-20260813-162941.jsonl, 21 questions x 1 repeat) to test whether the 2500 cap was the cause. It was not. Truncation fell from 31/42 to 3/21 and empty answers from 31 to 3, so the cap was a real constraint — but tool calls stayed at ZERO and the score did not move. Every run is one iteration: no tool call means nothing to feed back. It writes an essay about calling tools instead (309,720 chars of reasoning vs 10,186 of answer) naming tools that mostly do not exist (search_film_by_title, get_rental_film_id). Wire at 6000: 25 tools sent, no tool_calls field, 11,497 chars of 'thinking', content ending '&lt;tool&gt;search_film_by_title&lt;/tool&gt;' — its own invented pseudo-syntax in the content channel. Also ignores Agent:Thinking=false entirely (reasoning in every iteration). Costs 50% more wall clock at the higher cap for an identical zero. The earlier 'untestable at this MaxOutputTokens' caveat is retired — the cap was hiding the failure, not causing it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Phi4</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>mini</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Q4_K_M</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="F21" s="16" t="n">
+        <v>45689</v>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>phi4-mini</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="11" t="inlineStr">
+        <is>
+          <t>runs-20260813-165949.jsonl</t>
+        </is>
+      </c>
+      <c r="J21" s="11" t="n">
+        <v>21</v>
+      </c>
+      <c r="K21" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" s="11" t="n">
+        <v>2289</v>
+      </c>
+      <c r="T21" s="11" t="n">
+        <v>113</v>
+      </c>
+      <c r="U21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA21" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ21" s="8" t="inlineStr">
+        <is>
+          <t>HARD FAIL — zero tool calls in all 21 runs, wire-confirmed. True score 0/21: the single 'correct' is the same planning-monologue false positive as deepseek-r1. NOTE THE DIFFERENT CONFIG: Repeats=1 (21 runs, not 42) and MaxOutputTokens 6000, so the counts here are not directly comparable with the rows above; the rates are. Distinct from the other zero-call failures and the closest call of the four: it emits STRUCTURALLY CORRECT tool-call JSON — [{"name": "get_film", "arguments": {"film_id": 1}}] — with real tool and parameter names, but into the content channel (15 of 21 runs). Checked properly because that shape suggests a rig fault: /api/show reports phi4-mini declares the 'tools' capability and its template does handle them, rendering tools into &lt;|tool|&gt;...&lt;|/tool|&gt; and expecting calls back wrapped as &lt;|tool_call|&gt;[...]&lt;|/tool_call|&gt;. Wire capture: 25 tools sent, no tool_calls field in the response, and the content carries the bare JSON array with NO &lt;|tool_call|&gt; delimiter. So the model omits the delimiter its own chat template requires and Ollama cannot parse the payload — a model failure, but one pair of tags away from working. Two aggravating factors: it also hallucinates the RESULTS, roleplaying whole conversations with invented rows (invents the city 'Springfield', invents actor ids [1,2,3] then concludes '3 actors'), and its text-format calls are frequently malformed anyway ({"arguments"} as a second object rather than a key; "parameters" instead of "arguments"). Invents tools that do not exist (search_rental, search_inventory_item). Fast and cheap at 113 output tokens and 2.0s per run, which buys nothing.</t>
         </is>
       </c>
     </row>
@@ -3815,48 +3939,80 @@
       </c>
     </row>
     <row r="36">
-      <c r="H36" s="11" t="n"/>
+      <c r="G36" s="11" t="inlineStr">
+        <is>
+          <t>deepseek-r1:8b</t>
+        </is>
+      </c>
+      <c r="H36" s="11" t="inlineStr">
+        <is>
+          <t>Retested at MaxOutputTokens 6000: still zero tool calls. Reclassified as a hard fail alongside granite3.3:8b and command-r7b — all wire-confirmed to receive 25 tool definitions and call none.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="G37" s="10" t="inlineStr">
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t>phi4-mini</t>
+        </is>
+      </c>
+      <c r="H37" s="11" t="inlineStr">
+        <is>
+          <t>Zero tool calls, but emits well-formed tool-call JSON into the content channel without the &lt;|tool_call|&gt; delimiter its own template requires. Run at Repeats=1 / cap 6000, so 21 runs not 42.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="G38" s="11" t="n"/>
+      <c r="H38" s="11" t="n"/>
+    </row>
+    <row r="39">
+      <c r="G39" s="10" t="inlineStr">
         <is>
           <t>Validation</t>
         </is>
       </c>
-      <c r="H37" s="11" t="n"/>
-    </row>
-    <row r="38">
-      <c r="H38" s="11" t="inlineStr">
-        <is>
-          <t>All 22 rows recomputed from the regraded JSONL (grader deterministic-substring-v3). One transcription error found and corrected: ref /8 for qwen2.5:7b, 5 -&gt; 8.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="H39" s="11" t="inlineStr">
-        <is>
-          <t>v3 changes: fabricated arguments split into invented row id vs invented search term, and an answer truncated by the token cap can no longer be graded as a refusal. Regrading all 968 runs produced 0 correct/declined flips — both changes are additive.</t>
-        </is>
-      </c>
+      <c r="H39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>Caveat on the hop columns: the v2 near-miss and truncation questions all sit at hop 2, so 'hop 2 ans' measures search recovery as much as depth. Chain-only scores are in RESULTS-ANALYSIS.md.</t>
+          <t>All rows recomputed from the regraded JSONL (grader deterministic-substring-v3). One transcription error found and corrected: ref /8 for qwen2.5:7b, 5 -&gt; 8.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="H41" s="11" t="inlineStr">
         <is>
-          <t>Determinism check: 10 eval invocations of nearmiss-film-rate on qwen3.5:9b (20 runs) gave 19 bit-identical and 1 divergent only in the final free-text iteration; load_duration flat 238-324ms throughout, so not a model reload.</t>
+          <t>v3 changes: fabricated arguments split into invented row id vs invented search term, and an answer truncated by the token cap can no longer be graded as a refusal. Regrading all 968 runs produced 0 correct/declined flips — both changes are additive.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>gpt-5.6-sol and gpt-5.6-terra were run later, on the same config (standard+desc, seed 42, temp 0, repeats 2, thinking off, 2500 max tokens, v1+v2) and graded live at v3. One config difference from the earlier GPT rows: the OpenAI client now retries 429/5xx with backoff, which affects resilience, not output.</t>
+          <t>Caveat on the hop columns: the v2 near-miss and truncation questions all sit at hop 2, so 'hop 2 ans' measures search recovery as much as depth. Chain-only scores are in RESULTS-ANALYSIS.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="H43" s="11" t="inlineStr">
+        <is>
+          <t>Determinism check: 10 eval invocations of nearmiss-film-rate on qwen3.5:9b (20 runs) gave 19 bit-identical and 1 divergent only in the final free-text iteration; load_duration flat 238-324ms throughout, so not a model reload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="H44" s="11" t="inlineStr">
+        <is>
+          <t>gpt-5.6-sol and gpt-5.6-terra were run later on the same config and graded live at v3. One config difference from the earlier GPT rows: the OpenAI client now retries 429/5xx with backoff, which affects resilience, not output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>phi4-mini (row 21) and the deepseek-r1 retest used Repeats=1 and MaxOutputTokens 6000. Their run COUNTS are therefore out of 21, not 42; rates are comparable, totals are not.</t>
         </is>
       </c>
     </row>

</xml_diff>